<commit_message>
chore(RM-STAB-002): done — подтверждено прогоном CI, behavioral 475 passed
Прогон 33015298420 на 1e7a2bf — success, 0 провалов. Behavioral 475 passed
(470 прежних + 5 новых пинов strictness), governance guard 34/34 на раннере,
release-gate success.

Очередь: 43 задачи, done=9, planned=34. Следующая по этапу S — RM-STAB-003
(зафиксировать approved personas/retailer-scope, owner_gate scope_decision).

Поправка: номер 33014139714, названный в отчёте новым, был прогоном старого
коммита 3882592 — список взят до регистрации нового прогона.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCmxJQqxYurcepdgUpTP1p
</commit_message>
<xml_diff>
--- a/docs/product/generated/roadmap.generated.xlsx
+++ b/docs/product/generated/roadmap.generated.xlsx
@@ -1015,7 +1015,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>verification</t>
+          <t>done</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
@@ -1026,12 +1026,12 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>verified · behavioral · tests/behavioral/test_rls_context_strictness.py; verified · behavioral · RUN_BEHAVIORAL_TESTS=1 python3 -m pytest tests/behavioral -q; verified · behavioral · tamper — маска возвращена, хук фазы убран, запись allowlist без дефекта; verified · artifact · docs/architecture/rm-stab-002-strict-rls-context-design-gate.md</t>
+          <t>verified · behavioral · tests/behavioral/test_rls_context_strictness.py; verified · behavioral · RUN_BEHAVIORAL_TESTS=1 python3 -m pytest tests/behavioral -q; verified · behavioral · tamper — маска возвращена, хук фазы убран, запись allowlist без дефекта; verified · ci_run · gh run 33015298420 — Behavioral PostgreSQL Tests success на 1e7a2bf; verified · artifact · docs/architecture/rm-stab-002-strict-rls-context-design-gate.md</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>полная приёмка — docs/audit/2026-08-26-roadmap-task-breakdown-final-candidate.md (+v2); закрывает мою находку BEHAVIORAL-ADMIN-MASK-001. Элевация привязана к фазе прогона: setup и teardown элевированы, тело теста strict. Замер показал, что на маске держались 181 из 470 тестов — 148 setup, 13 teardown, 20 тел. Вскрыт продовый дефект на двух device-маршрутах; по решению владельца вынесен в отдельную задачу RM-TECH-210, обе записи allowlist названы поимённо и снимаются её починкой.</t>
+          <t>полная приёмка — docs/audit/2026-08-26-roadmap-task-breakdown-final-candidate.md (+v2); закрывает мою находку BEHAVIORAL-ADMIN-MASK-001. Элевация привязана к фазе прогона. Замер: на маске держались 181 из 470 тестов — 148 setup, 13 teardown, 20 тел. Вскрыт продовый дефект на двух device-маршрутах, по решению владельца вынесен в RM-TECH-210. Подтверждено на раннере прогоном 33015298420: behavioral 475 passed (470 прежних + 5 новых пинов), release-gate success.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
governance(RM-GOV-009): evidence CI run 33169752021 (2b7713e success) — 64 задачи approved, RM-GOV-009 verification
Владелец 2026-08-28 принял очередь A3: decision_status proposed → approved у 64 задач
(потолок approved; done — только отдельным ACCEPT). RM-GOV-009 → verification с ci_run
evidence. Delivery-статусы не менялись. Проекции регенерированы; PROJECT_STATE и запись
docs/audit/2026-08-28-claude-rm-gov-009-applied.md §7.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCmxJQqxYurcepdgUpTP1p
</commit_message>
<xml_diff>
--- a/docs/product/generated/roadmap.generated.xlsx
+++ b/docs/product/generated/roadmap.generated.xlsx
@@ -894,7 +894,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -950,7 +950,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1006,12 +1006,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>planned</t>
+          <t>verification</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>verified · ci_run · https://github.com/santanas-dev/retail-media-platform-enterprise/actions/runs/33169752021</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2154,7 +2154,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -2898,7 +2898,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -3346,7 +3346,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -3574,7 +3574,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -3802,7 +3802,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -3858,7 +3858,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -4030,7 +4030,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
@@ -4710,7 +4710,7 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
@@ -4822,7 +4822,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -5058,7 +5058,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -5118,7 +5118,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -5178,7 +5178,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -5234,7 +5234,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -5346,7 +5346,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -5574,7 +5574,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -5634,7 +5634,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -5690,7 +5690,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -5746,7 +5746,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
@@ -5806,7 +5806,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -5862,7 +5862,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -5918,7 +5918,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -6030,7 +6030,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -6086,7 +6086,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -6142,7 +6142,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>approved</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">

</xml_diff>